<commit_message>
Added import logic and example for owned subnets
</commit_message>
<xml_diff>
--- a/example_data.xlsx
+++ b/example_data.xlsx
@@ -18,6 +18,10 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="VLAN_500_Guest-Wifi" sheetId="9" state="visible" r:id="rId9"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="VLAN_600_Colo-Hosting" sheetId="10" state="visible" r:id="rId10"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="VLAN_700_Backup-Net" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="VLAN_800_Public-Web" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="VLAN_810_Cust-Widgets" sheetId="13" state="visible" r:id="rId13"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="VLAN_999_Transit" sheetId="14" state="visible" r:id="rId14"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Owned_Subnets" sheetId="15" state="visible" r:id="rId15"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -6075,6 +6079,1844 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:I28"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="15" customWidth="1" min="1" max="1"/>
+    <col width="15" customWidth="1" min="2" max="2"/>
+    <col width="15" customWidth="1" min="3" max="3"/>
+    <col width="15" customWidth="1" min="4" max="4"/>
+    <col width="15" customWidth="1" min="5" max="5"/>
+    <col width="15" customWidth="1" min="6" max="6"/>
+    <col width="15" customWidth="1" min="7" max="7"/>
+    <col width="15" customWidth="1" min="8" max="8"/>
+    <col width="15" customWidth="1" min="9" max="9"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>VLAN Metadata</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>VLAN 800</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>Name: Public-Web</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>Routed: Yes</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>Uplink: FW-Ext Gi0/1</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>Customer: Acme Corp</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>Location: DC-East-1</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>Comment: Public-facing services (NAT + direct)</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>Subnet Name</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>CIDR</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="inlineStr">
+        <is>
+          <t>IP Address</t>
+        </is>
+      </c>
+      <c r="D3" s="2" t="inlineStr">
+        <is>
+          <t>Customer</t>
+        </is>
+      </c>
+      <c r="E3" s="2" t="inlineStr">
+        <is>
+          <t>Location</t>
+        </is>
+      </c>
+      <c r="F3" s="2" t="inlineStr">
+        <is>
+          <t>Comment</t>
+        </is>
+      </c>
+      <c r="G3" s="2" t="inlineStr">
+        <is>
+          <t>Asset</t>
+        </is>
+      </c>
+      <c r="H3" s="2" t="inlineStr">
+        <is>
+          <t>Interface</t>
+        </is>
+      </c>
+      <c r="I3" s="2" t="inlineStr">
+        <is>
+          <t>Network Connection</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Web-Public</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>203.0.113.0/27</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>203.0.113.1</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>Acme Corp</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>DC-East-1</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>Gateway</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>Palo Alto PA-5260</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>Gi0/1</t>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>Direct to Firewall</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Web-Public</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>203.0.113.0/27</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>203.0.113.2</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>Acme Corp</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>DC-East-1</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>nginx-prod-01</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>Dell R740</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>eth0</t>
+        </is>
+      </c>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>LACP to TOR-A</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Web-Public</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>203.0.113.0/27</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>203.0.113.3</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>Acme Corp</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>DC-East-1</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>nginx-prod-02</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>Dell R740</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>eth0</t>
+        </is>
+      </c>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>LACP to TOR-A</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Web-Public</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>203.0.113.0/27</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>203.0.113.4</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>Acme Corp</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>DC-East-1</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>nginx-prod-03</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>Dell R740</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>eth0</t>
+        </is>
+      </c>
+      <c r="I7" t="inlineStr">
+        <is>
+          <t>LACP to TOR-B</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Web-Public</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>203.0.113.0/27</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>203.0.113.5</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>Acme Corp</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>DC-East-1</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>HAProxy VIP - primary</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>F5 BIG-IP i5800</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>bond0</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Web-Public</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>203.0.113.0/27</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>203.0.113.6</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>Acme Corp</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>DC-East-1</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>HAProxy VIP - standby</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>F5 BIG-IP i5800</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>bond0</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Web-Public</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>203.0.113.0/27</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>203.0.113.7</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>Globex Industries</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>DC-East-1</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>Customer portal</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>Ubuntu 22.04 LTS</t>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>ens192</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Web-Public</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>203.0.113.0/27</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>203.0.113.8</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>Acme Corp</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>DC-East-1</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>API gateway</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>K8s Worker Node</t>
+        </is>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>eth0</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>Web-Public</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>203.0.113.0/27</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>203.0.113.9</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>Acme Corp</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>DC-East-1</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>Webhook receiver</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>Docker Host</t>
+        </is>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>eth0</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>Web-Public</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>203.0.113.0/27</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>203.0.113.10</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>Acme Corp</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>DC-East-1</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>Status page (Cachet)</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>Ubuntu 22.04 LTS</t>
+        </is>
+      </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>ens192</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>Web-Public</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>203.0.113.0/27</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>203.0.113.11</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>Oscorp Data</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>DC-East-1</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>Customer API endpoint</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>RHEL 9 Server</t>
+        </is>
+      </c>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>bond0</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>Web-Public</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>203.0.113.0/27</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>203.0.113.12</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>Acme Corp</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>DC-East-1</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>Scheduled for decom Q3</t>
+        </is>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>Cisco C220 M5</t>
+        </is>
+      </c>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t>eth0</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>Web-Public</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>203.0.113.0/27</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>203.0.113.15</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>Acme Corp</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>DC-East-1</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>mail relay outbound</t>
+        </is>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>Ubuntu 22.04 LTS</t>
+        </is>
+      </c>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t>ens192</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>Web-Public</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>203.0.113.0/27</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>203.0.113.20</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>Acme Corp</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>Monitoring probe</t>
+        </is>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>Raspberry Pi 4</t>
+        </is>
+      </c>
+      <c r="H17" t="inlineStr">
+        <is>
+          <t>eth0</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>Mail-Public</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>203.0.113.32/29</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>203.0.113.33</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>Acme Corp</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>DC-East-1</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>Gateway</t>
+        </is>
+      </c>
+      <c r="H18" t="inlineStr">
+        <is>
+          <t>Gi0/2</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>Mail-Public</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>203.0.113.32/29</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>203.0.113.34</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>Acme Corp</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>DC-East-1</t>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>MX primary</t>
+        </is>
+      </c>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>HP DL360 Gen10</t>
+        </is>
+      </c>
+      <c r="H19" t="inlineStr">
+        <is>
+          <t>eth0</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>Mail-Public</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>203.0.113.32/29</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>203.0.113.35</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>Acme Corp</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>DC-East-1</t>
+        </is>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>MX secondary</t>
+        </is>
+      </c>
+      <c r="G20" t="inlineStr">
+        <is>
+          <t>HP DL360 Gen10</t>
+        </is>
+      </c>
+      <c r="H20" t="inlineStr">
+        <is>
+          <t>eth0</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>Mail-Public</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>203.0.113.32/29</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>203.0.113.36</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>Acme Corp</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>DC-East-1</t>
+        </is>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>SMTP relay</t>
+        </is>
+      </c>
+      <c r="G21" t="inlineStr">
+        <is>
+          <t>Ubuntu 22.04 LTS</t>
+        </is>
+      </c>
+      <c r="H21" t="inlineStr">
+        <is>
+          <t>ens192</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>Mail-Public</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>203.0.113.32/29</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>203.0.113.37</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>Acme Corp</t>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>DC-East-1</t>
+        </is>
+      </c>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>SPF/DKIM signer</t>
+        </is>
+      </c>
+      <c r="G22" t="inlineStr">
+        <is>
+          <t>Ubuntu 22.04 LTS</t>
+        </is>
+      </c>
+      <c r="H22" t="inlineStr">
+        <is>
+          <t>ens192</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>Mail-Public</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>203.0.113.32/29</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>203.0.113.38</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>Acme Corp</t>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>DC-East-1</t>
+        </is>
+      </c>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>Spam filter</t>
+        </is>
+      </c>
+      <c r="G23" t="inlineStr">
+        <is>
+          <t>Cisco C220 M5</t>
+        </is>
+      </c>
+      <c r="H23" t="inlineStr">
+        <is>
+          <t>eth0</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>VPN-Endpoints</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>203.0.113.64/28</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>203.0.113.65</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>Acme Corp</t>
+        </is>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>DC-East-1</t>
+        </is>
+      </c>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t>Gateway</t>
+        </is>
+      </c>
+      <c r="H24" t="inlineStr">
+        <is>
+          <t>Gi0/3</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>VPN-Endpoints</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>203.0.113.64/28</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>203.0.113.66</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>Acme Corp</t>
+        </is>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>DC-East-1</t>
+        </is>
+      </c>
+      <c r="F25" t="inlineStr">
+        <is>
+          <t>IPSec concentrator</t>
+        </is>
+      </c>
+      <c r="G25" t="inlineStr">
+        <is>
+          <t>Palo Alto PA-5260</t>
+        </is>
+      </c>
+      <c r="H25" t="inlineStr">
+        <is>
+          <t>eth1</t>
+        </is>
+      </c>
+      <c r="I25" t="inlineStr">
+        <is>
+          <t>Internet edge</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>VPN-Endpoints</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>203.0.113.64/28</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>203.0.113.67</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>Acme Corp</t>
+        </is>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>DC-East-1</t>
+        </is>
+      </c>
+      <c r="F26" t="inlineStr">
+        <is>
+          <t>WireGuard endpoint</t>
+        </is>
+      </c>
+      <c r="G26" t="inlineStr">
+        <is>
+          <t>Ubuntu 22.04 LTS</t>
+        </is>
+      </c>
+      <c r="H26" t="inlineStr">
+        <is>
+          <t>wg0</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>VPN-Endpoints</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>203.0.113.64/28</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>203.0.113.70</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>Acme Corp</t>
+        </is>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>DC-East-1</t>
+        </is>
+      </c>
+      <c r="F27" t="inlineStr">
+        <is>
+          <t>Site-to-site - Chicago</t>
+        </is>
+      </c>
+      <c r="I27" t="inlineStr">
+        <is>
+          <t>MPLS PE link</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>VPN-Endpoints</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>203.0.113.64/28</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>203.0.113.71</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>Acme Corp</t>
+        </is>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>DC-East-1</t>
+        </is>
+      </c>
+      <c r="F28" t="inlineStr">
+        <is>
+          <t>Site-to-site - Denver</t>
+        </is>
+      </c>
+      <c r="I28" t="inlineStr">
+        <is>
+          <t>MPLS PE link</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:I8"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="15" customWidth="1" min="1" max="1"/>
+    <col width="15" customWidth="1" min="2" max="2"/>
+    <col width="15" customWidth="1" min="3" max="3"/>
+    <col width="15" customWidth="1" min="4" max="4"/>
+    <col width="15" customWidth="1" min="5" max="5"/>
+    <col width="15" customWidth="1" min="6" max="6"/>
+    <col width="15" customWidth="1" min="7" max="7"/>
+    <col width="15" customWidth="1" min="8" max="8"/>
+    <col width="15" customWidth="1" min="9" max="9"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>VLAN Metadata</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>VLAN 810</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>Name: Cust-Widgets</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>Routed: Yes</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>Uplink: FW-Ext Gi0/3</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>Customer: Widgets Inc</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>Location: DC-East-1 Cage 7</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>Comment: Dedicated customer allocation</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>Subnet Name</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>CIDR</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="inlineStr">
+        <is>
+          <t>IP Address</t>
+        </is>
+      </c>
+      <c r="D3" s="2" t="inlineStr">
+        <is>
+          <t>Customer</t>
+        </is>
+      </c>
+      <c r="E3" s="2" t="inlineStr">
+        <is>
+          <t>Location</t>
+        </is>
+      </c>
+      <c r="F3" s="2" t="inlineStr">
+        <is>
+          <t>Comment</t>
+        </is>
+      </c>
+      <c r="G3" s="2" t="inlineStr">
+        <is>
+          <t>Asset</t>
+        </is>
+      </c>
+      <c r="H3" s="2" t="inlineStr">
+        <is>
+          <t>Interface</t>
+        </is>
+      </c>
+      <c r="I3" s="2" t="inlineStr">
+        <is>
+          <t>Network Connection</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Widgets-Servers</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>203.0.113.128/26</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>203.0.113.129</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>Widgets Inc</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>DC-East-1 Cage 7</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>Gateway</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>Gi0/0</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Widgets-Servers</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>203.0.113.128/26</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>203.0.113.130</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>Widgets Inc</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>DC-East-1 Cage 7</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>Customer web server</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>Dell R640</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>eth0</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Widgets-Servers</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>203.0.113.128/26</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>203.0.113.131</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>Widgets Inc</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>DC-East-1 Cage 7</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>Customer API</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>Dell R640</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>eth0</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Widgets-Servers</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>203.0.113.128/26</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>203.0.113.132</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>Widgets Inc</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>DC-East-1 Cage 7</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>Customer DB</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>Dell R740</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>eth0</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Widgets-Servers</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>203.0.113.128/26</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>203.0.113.135</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>Widgets Inc</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>DC-East-1 Cage 7</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>Monitoring</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>Raspberry Pi 4</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>eth0</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:I7"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="15" customWidth="1" min="1" max="1"/>
+    <col width="15" customWidth="1" min="2" max="2"/>
+    <col width="15" customWidth="1" min="3" max="3"/>
+    <col width="15" customWidth="1" min="4" max="4"/>
+    <col width="15" customWidth="1" min="5" max="5"/>
+    <col width="15" customWidth="1" min="6" max="6"/>
+    <col width="15" customWidth="1" min="7" max="7"/>
+    <col width="15" customWidth="1" min="8" max="8"/>
+    <col width="15" customWidth="1" min="9" max="9"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>VLAN Metadata</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>VLAN 999</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>Name: Transit</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>Routed: Yes</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Uplink: </t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Customer: </t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>Location: DC-East-1 MDF</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>Comment: Upstream transit point-to-point links</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>Subnet Name</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>CIDR</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="inlineStr">
+        <is>
+          <t>IP Address</t>
+        </is>
+      </c>
+      <c r="D3" s="2" t="inlineStr">
+        <is>
+          <t>Customer</t>
+        </is>
+      </c>
+      <c r="E3" s="2" t="inlineStr">
+        <is>
+          <t>Location</t>
+        </is>
+      </c>
+      <c r="F3" s="2" t="inlineStr">
+        <is>
+          <t>Comment</t>
+        </is>
+      </c>
+      <c r="G3" s="2" t="inlineStr">
+        <is>
+          <t>Asset</t>
+        </is>
+      </c>
+      <c r="H3" s="2" t="inlineStr">
+        <is>
+          <t>Interface</t>
+        </is>
+      </c>
+      <c r="I3" s="2" t="inlineStr">
+        <is>
+          <t>Network Connection</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Cogent-Uplink</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>198.51.100.0/30</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>198.51.100.1</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>Soylent ISP</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>DC-East-1 MDF</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>Our side - Cogent</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>Cisco ASR 9001</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>Gi0/0/0</t>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>Cross-connect to Meet-Me</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Cogent-Uplink</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>198.51.100.0/30</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>198.51.100.2</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>Soylent ISP</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>DC-East-1 MDF</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>Cogent PE router</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>et-0/0/1</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Lumen-Uplink</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>198.51.100.4/30</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>198.51.100.5</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>Soylent ISP</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>DC-East-1 MDF</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>Our side - Lumen</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>Cisco ASR 9001</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>Gi0/0/1</t>
+        </is>
+      </c>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>Cross-connect to Meet-Me</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Lumen-Uplink</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>198.51.100.4/30</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>198.51.100.6</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>Soylent ISP</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>DC-East-1 MDF</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>Lumen PE router</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:B5"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="22" customWidth="1" min="1" max="1"/>
+    <col width="45" customWidth="1" min="2" max="2"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="2" t="inlineStr">
+        <is>
+          <t>CIDR</t>
+        </is>
+      </c>
+      <c r="B1" s="2" t="inlineStr">
+        <is>
+          <t>Label</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>203.0.113.0/24</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Cogent Allocation - Jan 2023</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>198.51.100.0/28</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Transit Block - Soylent ISP</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>192.0.2.0/24</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>ARIN Transfer - Dec 2024 (staging)</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>198.18.128.0/25</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Customer Block - Reserved for Initech</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>

</xml_diff>